<commit_message>
Week 5 results and name updates
</commit_message>
<xml_diff>
--- a/FFL_Data.xlsx
+++ b/FFL_Data.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://claycorp-my.sharepoint.com/personal/axelrade_claycorp_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\axelrade\Downloads\FFL-Dash-2026-main\FFL-Dash-2026-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{93964692-C241-4089-85D1-8F0C2ABFCCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23948E8E-B573-466D-ABAE-EFC404220FD1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCD3205-2497-4F29-BEE1-16E7D62AB102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Weekly Results" sheetId="1" r:id="rId1"/>
+    <sheet name="2026 Results" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Weekly Results'!$A$1:$E$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026 Results'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="35">
   <si>
     <t>Team</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Points Against</t>
   </si>
   <si>
-    <t>Projected Points For</t>
-  </si>
-  <si>
     <t>Dicker in LaPorta</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
     <t>Mucha Novias Mucha Piñeiros</t>
   </si>
   <si>
-    <t>Quad Goals</t>
-  </si>
-  <si>
     <t>Stern but Fairbairn</t>
   </si>
   <si>
@@ -138,13 +132,22 @@
   </si>
   <si>
     <t>Team Icons/vele-modified.png</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Projected Points</t>
+  </si>
+  <si>
+    <t>Laffy Taffy McCaffrey</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,10 +168,14 @@
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
+      <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -207,7 +214,7 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -534,18 +541,18 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="4">
         <v>114.3</v>
@@ -559,10 +566,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4">
         <v>143.5</v>
@@ -576,10 +583,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="4">
         <v>110.02</v>
@@ -593,10 +600,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="4">
         <v>120.66</v>
@@ -610,95 +617,95 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="4">
+        <v>77.260000000000005</v>
+      </c>
+      <c r="D6" s="4">
         <v>131.56</v>
       </c>
-      <c r="D6" s="4">
-        <v>77.260000000000005</v>
-      </c>
       <c r="E6" s="4">
-        <v>107.5</v>
+        <v>97.23</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C7" s="4">
-        <v>99.06</v>
+        <v>131.56</v>
       </c>
       <c r="D7" s="4">
-        <v>110.02</v>
+        <v>77.260000000000005</v>
       </c>
       <c r="E7" s="4">
-        <v>109.01</v>
+        <v>107.5</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="4">
-        <v>95.72</v>
+        <v>99.06</v>
       </c>
       <c r="D8" s="4">
-        <v>120.66</v>
+        <v>110.02</v>
       </c>
       <c r="E8" s="4">
-        <v>108.63</v>
+        <v>109.01</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="4">
-        <v>142.34</v>
+        <v>95.72</v>
       </c>
       <c r="D9" s="4">
-        <v>114.3</v>
+        <v>120.66</v>
       </c>
       <c r="E9" s="4">
-        <v>108.62</v>
+        <v>108.63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C10" s="4">
-        <v>77.260000000000005</v>
+        <v>142.34</v>
       </c>
       <c r="D10" s="4">
-        <v>131.56</v>
+        <v>114.3</v>
       </c>
       <c r="E10" s="4">
-        <v>97.23</v>
+        <v>108.62</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C11" s="4">
         <v>101.06</v>
@@ -712,10 +719,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C12" s="4">
         <v>114.76</v>
@@ -729,10 +736,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="C13" s="4">
         <v>122.8</v>
@@ -746,10 +753,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14" s="4">
         <v>137.47999999999999</v>
@@ -763,10 +770,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15" s="4">
         <v>107.06</v>
@@ -780,10 +787,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16" s="4">
         <v>75.06</v>
@@ -797,10 +804,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C17" s="4">
         <v>63.72</v>
@@ -814,95 +821,95 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C18" s="4">
-        <v>92</v>
+        <v>98.34</v>
       </c>
       <c r="D18" s="4">
-        <v>107.58</v>
+        <v>119.86</v>
       </c>
       <c r="E18" s="4">
-        <v>109.24</v>
+        <v>111.15</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C19" s="4">
-        <v>114.02</v>
+        <v>92</v>
       </c>
       <c r="D19" s="4">
-        <v>107.06</v>
+        <v>107.58</v>
       </c>
       <c r="E19" s="4">
-        <v>114.75</v>
+        <v>109.24</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C20" s="4">
-        <v>115.12</v>
+        <v>114.02</v>
       </c>
       <c r="D20" s="4">
-        <v>101.98</v>
+        <v>107.06</v>
       </c>
       <c r="E20" s="4">
-        <v>107.77</v>
+        <v>114.75</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C21" s="4">
+        <v>115.12</v>
+      </c>
+      <c r="D21" s="4">
         <v>101.98</v>
       </c>
-      <c r="D21" s="4">
-        <v>115.12</v>
-      </c>
       <c r="E21" s="4">
-        <v>107.54</v>
+        <v>107.77</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C22" s="4">
-        <v>98.34</v>
+        <v>101.98</v>
       </c>
       <c r="D22" s="4">
-        <v>119.86</v>
+        <v>115.12</v>
       </c>
       <c r="E22" s="4">
-        <v>111.15</v>
+        <v>107.54</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C23" s="4">
         <v>101.08</v>
@@ -916,10 +923,10 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C24" s="4">
         <v>107.58</v>
@@ -933,10 +940,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C25" s="4">
         <v>119.86</v>
@@ -950,10 +957,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C26" s="4">
         <v>133.19999999999999</v>
@@ -967,10 +974,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C27" s="4">
         <v>96.98</v>
@@ -984,10 +991,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C28" s="4">
         <v>106.54</v>
@@ -1001,10 +1008,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C29" s="4">
         <v>94.1</v>
@@ -1018,95 +1025,95 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C30" s="4">
-        <v>169.14</v>
+        <v>116.46</v>
       </c>
       <c r="D30" s="4">
-        <v>133.19999999999999</v>
+        <v>111.74</v>
       </c>
       <c r="E30" s="4">
-        <v>114.4</v>
+        <v>101.96</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C31" s="4">
-        <v>105.86</v>
+        <v>169.14</v>
       </c>
       <c r="D31" s="4">
-        <v>95.04</v>
+        <v>133.19999999999999</v>
       </c>
       <c r="E31" s="4">
-        <v>112.19</v>
+        <v>114.4</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="4">
+        <v>105.86</v>
+      </c>
+      <c r="D32" s="4">
+        <v>95.04</v>
+      </c>
+      <c r="E32" s="4">
+        <v>112.19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="4">
+        <v>77.86</v>
+      </c>
+      <c r="D33" s="4">
+        <v>111.28</v>
+      </c>
+      <c r="E33" s="4">
+        <v>98.97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="4">
-        <v>77.86</v>
-      </c>
-      <c r="D32" s="4">
-        <v>111.28</v>
-      </c>
-      <c r="E32" s="4">
-        <v>98.97</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="B34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="4">
+        <v>83.36</v>
+      </c>
+      <c r="D34" s="4">
+        <v>106.54</v>
+      </c>
+      <c r="E34" s="4">
+        <v>107.3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="4">
-        <v>83.36</v>
-      </c>
-      <c r="D33" s="4">
-        <v>106.54</v>
-      </c>
-      <c r="E33" s="4">
-        <v>107.3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="4">
-        <v>116.46</v>
-      </c>
-      <c r="D34" s="4">
-        <v>111.74</v>
-      </c>
-      <c r="E34" s="4">
-        <v>101.96</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="B35" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C35" s="4">
         <v>111.28</v>
@@ -1118,12 +1125,12 @@
         <v>96.4</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C36" s="4">
         <v>111.74</v>
@@ -1135,12 +1142,12 @@
         <v>106.37</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C37" s="4">
         <v>95.04</v>
@@ -1152,12 +1159,12 @@
         <v>107.34</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C38" s="4">
         <v>100.48</v>
@@ -1168,16 +1175,13 @@
       <c r="E38" s="4">
         <v>111.92</v>
       </c>
-      <c r="F38" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C39" s="4">
         <v>73.58</v>
@@ -1188,16 +1192,13 @@
       <c r="E39" s="4">
         <v>103.86</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C40" s="4">
         <v>106.6</v>
@@ -1208,16 +1209,13 @@
       <c r="E40" s="4">
         <v>107.38</v>
       </c>
-      <c r="F40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C41" s="4">
         <v>76.040000000000006</v>
@@ -1228,116 +1226,98 @@
       <c r="E41" s="4">
         <v>109.59</v>
       </c>
-      <c r="F41" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="4">
+        <v>104.22</v>
+      </c>
+      <c r="D42" s="4">
+        <v>100.48</v>
+      </c>
+      <c r="E42" s="4">
+        <v>107.46</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" s="4">
+        <v>103.78</v>
+      </c>
+      <c r="D43" s="4">
+        <v>156.46</v>
+      </c>
+      <c r="E43" s="4">
+        <v>118.34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42" s="4">
+      <c r="B44" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" s="4">
+        <v>55.32</v>
+      </c>
+      <c r="D44" s="4">
+        <v>76.040000000000006</v>
+      </c>
+      <c r="E44" s="4">
+        <v>100.07</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="4">
+        <v>156.46</v>
+      </c>
+      <c r="D45" s="4">
         <v>103.78</v>
       </c>
-      <c r="D42" s="4">
-        <v>156.46</v>
-      </c>
-      <c r="E42" s="4">
-        <v>118.34</v>
-      </c>
-      <c r="F42" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43" s="4">
-        <v>55.32</v>
-      </c>
-      <c r="D43" s="4">
-        <v>76.040000000000006</v>
-      </c>
-      <c r="E43" s="4">
-        <v>100.07</v>
-      </c>
-      <c r="F43" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="E45" s="4">
+        <v>105.81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44" s="4">
-        <v>156.46</v>
-      </c>
-      <c r="D44" s="4">
-        <v>103.78</v>
-      </c>
-      <c r="E44" s="4">
-        <v>105.81</v>
-      </c>
-      <c r="F44" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+      <c r="B46" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" s="4">
+        <v>120.98</v>
+      </c>
+      <c r="D46" s="4">
+        <v>73.58</v>
+      </c>
+      <c r="E46" s="4">
+        <v>117.49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45" s="4">
-        <v>120.98</v>
-      </c>
-      <c r="D45" s="4">
-        <v>73.58</v>
-      </c>
-      <c r="E45" s="4">
-        <v>117.49</v>
-      </c>
-      <c r="F45" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C46" s="4">
-        <v>104.22</v>
-      </c>
-      <c r="D46" s="4">
-        <v>100.48</v>
-      </c>
-      <c r="E46" s="4">
-        <v>107.46</v>
-      </c>
-      <c r="F46" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="B47" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C47" s="4">
         <v>112.02</v>
@@ -1348,16 +1328,13 @@
       <c r="E47" s="4">
         <v>108.97</v>
       </c>
-      <c r="F47" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C48" s="4">
         <v>168.48</v>
@@ -1368,16 +1345,13 @@
       <c r="E48" s="4">
         <v>114.89</v>
       </c>
-      <c r="F48" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C49" s="4">
         <v>143.30000000000001</v>
@@ -1388,14 +1362,249 @@
       <c r="E49" s="4">
         <v>112.81</v>
       </c>
-      <c r="F49" t="s">
-        <v>33</v>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C50" s="6">
+        <v>140.12</v>
+      </c>
+      <c r="D50" s="6">
+        <v>128.74</v>
+      </c>
+      <c r="E50" s="6">
+        <v>121.81</v>
+      </c>
+      <c r="F50" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="5"/>
+      <c r="A51" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C51" s="6">
+        <v>108.34</v>
+      </c>
+      <c r="D51" s="6">
+        <v>126.1</v>
+      </c>
+      <c r="E51" s="6">
+        <v>101.2</v>
+      </c>
+      <c r="F51" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C52" s="6">
+        <v>123.8</v>
+      </c>
+      <c r="D52" s="6">
+        <v>85.66</v>
+      </c>
+      <c r="E52" s="6">
+        <v>105.49</v>
+      </c>
+      <c r="F52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C53" s="6">
+        <v>113.24</v>
+      </c>
+      <c r="D53" s="6">
+        <v>103.34</v>
+      </c>
+      <c r="E53" s="6">
+        <v>111.17</v>
+      </c>
+      <c r="F53" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C54" s="6">
+        <v>129.06</v>
+      </c>
+      <c r="D54" s="6">
+        <v>88.06</v>
+      </c>
+      <c r="E54" s="6">
+        <v>105.38</v>
+      </c>
+      <c r="F54" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C55" s="6">
+        <v>85.66</v>
+      </c>
+      <c r="D55" s="6">
+        <v>123.8</v>
+      </c>
+      <c r="E55" s="6">
+        <v>119.22</v>
+      </c>
+      <c r="F55" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" s="6">
+        <v>115.3</v>
+      </c>
+      <c r="D56" s="6">
+        <v>141.24</v>
+      </c>
+      <c r="E56" s="6">
+        <v>108.3</v>
+      </c>
+      <c r="F56" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="6">
+        <v>88.06</v>
+      </c>
+      <c r="D57" s="6">
+        <v>129.06</v>
+      </c>
+      <c r="E57" s="6">
+        <v>103.14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C58" s="6">
+        <v>141.24</v>
+      </c>
+      <c r="D58" s="6">
+        <v>115.3</v>
+      </c>
+      <c r="E58" s="6">
+        <v>117.67</v>
+      </c>
+      <c r="F58" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C59" s="6">
+        <v>126.1</v>
+      </c>
+      <c r="D59" s="6">
+        <v>108.34</v>
+      </c>
+      <c r="E59" s="6">
+        <v>107.35</v>
+      </c>
+      <c r="F59" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C60" s="6">
+        <v>128.74</v>
+      </c>
+      <c r="D60" s="6">
+        <v>140.12</v>
+      </c>
+      <c r="E60" s="6">
+        <v>105.91</v>
+      </c>
+      <c r="F60" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C61" s="6">
+        <v>103.34</v>
+      </c>
+      <c r="D61" s="6">
+        <v>113.24</v>
+      </c>
+      <c r="E61" s="6">
+        <v>105.37</v>
+      </c>
+      <c r="F61" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Week 6 updates to results and .Rmd
Updated the team icons and colors
</commit_message>
<xml_diff>
--- a/FFL_Data.xlsx
+++ b/FFL_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\axelrade\Downloads\FFL-Dash-2026-main\FFL-Dash-2026-main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edenaxelrad/Desktop/FF Weekly Results/FFL-Dash-2026-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCD3205-2497-4F29-BEE1-16E7D62AB102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CF0882-2CE0-1E49-B74B-9408DD4CCEAE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Results" sheetId="1" r:id="rId1"/>
@@ -18,25 +18,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026 Results'!$A$1:$F$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="36">
   <si>
     <t>Team</t>
   </si>
@@ -62,12 +49,6 @@
     <t>Jaggin Off</t>
   </si>
   <si>
-    <t>Lamar-a-Lago</t>
-  </si>
-  <si>
-    <t>Mevis and Butthead</t>
-  </si>
-  <si>
     <t>MonanGai Fieri</t>
   </si>
   <si>
@@ -110,21 +91,12 @@
     <t>Team Icons/jaggin-modified.png</t>
   </si>
   <si>
-    <t>Team Icons/lamar-modified.png</t>
-  </si>
-  <si>
-    <t>Team Icons/mevis-modified.png</t>
-  </si>
-  <si>
     <t>Team Icons/monangai-modified.png</t>
   </si>
   <si>
     <t>Team Icons/novias-modified.png</t>
   </si>
   <si>
-    <t>Team Icons/quad-modified.png</t>
-  </si>
-  <si>
     <t>Team Icons/stern-modified.png</t>
   </si>
   <si>
@@ -141,6 +113,24 @@
   </si>
   <si>
     <t>Laffy Taffy McCaffrey</t>
+  </si>
+  <si>
+    <t>Carry me Joshy</t>
+  </si>
+  <si>
+    <t>Charbmander</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Team Icons/joshy-modified.png</t>
+  </si>
+  <si>
+    <t>Team Icons/charb-modified.png</t>
+  </si>
+  <si>
+    <t>Team Icons/laffy-modified.png</t>
   </si>
 </sst>
 </file>
@@ -170,6 +160,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -517,8 +508,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F61"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -527,7 +518,7 @@
     <col min="5" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -541,18 +532,18 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C2" s="4">
         <v>114.3</v>
@@ -564,12 +555,12 @@
         <v>109.91</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3" s="4">
         <v>143.5</v>
@@ -581,12 +572,12 @@
         <v>104.59</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4">
         <v>110.02</v>
@@ -598,12 +589,12 @@
         <v>108.04</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4">
         <v>120.66</v>
@@ -615,12 +606,12 @@
         <v>111.11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="4">
         <v>77.260000000000005</v>
@@ -632,12 +623,12 @@
         <v>97.23</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" s="4">
         <v>131.56</v>
@@ -649,12 +640,12 @@
         <v>107.5</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" s="4">
         <v>99.06</v>
@@ -666,12 +657,12 @@
         <v>109.01</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C9" s="4">
         <v>95.72</v>
@@ -683,12 +674,12 @@
         <v>108.63</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" s="4">
         <v>142.34</v>
@@ -700,12 +691,12 @@
         <v>108.62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C11" s="4">
         <v>101.06</v>
@@ -717,12 +708,12 @@
         <v>108.37</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="4">
         <v>114.76</v>
@@ -734,12 +725,12 @@
         <v>104.87</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="C13" s="4">
         <v>122.8</v>
@@ -751,12 +742,12 @@
         <v>110.93</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" s="4">
         <v>137.47999999999999</v>
@@ -768,12 +759,12 @@
         <v>113.37</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C15" s="4">
         <v>107.06</v>
@@ -785,12 +776,12 @@
         <v>106.98</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C16" s="4">
         <v>75.06</v>
@@ -802,12 +793,12 @@
         <v>98.07</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="4">
         <v>63.72</v>
@@ -819,12 +810,12 @@
         <v>104.97</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C18" s="4">
         <v>98.34</v>
@@ -836,12 +827,12 @@
         <v>111.15</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C19" s="4">
         <v>92</v>
@@ -853,12 +844,12 @@
         <v>109.24</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C20" s="4">
         <v>114.02</v>
@@ -870,12 +861,12 @@
         <v>114.75</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C21" s="4">
         <v>115.12</v>
@@ -887,12 +878,12 @@
         <v>107.77</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C22" s="4">
         <v>101.98</v>
@@ -904,12 +895,12 @@
         <v>107.54</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C23" s="4">
         <v>101.08</v>
@@ -921,12 +912,12 @@
         <v>103.51</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C24" s="4">
         <v>107.58</v>
@@ -938,12 +929,12 @@
         <v>106.49</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C25" s="4">
         <v>119.86</v>
@@ -955,12 +946,12 @@
         <v>106.43</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C26" s="4">
         <v>133.19999999999999</v>
@@ -972,12 +963,12 @@
         <v>108.84</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C27" s="4">
         <v>96.98</v>
@@ -989,12 +980,12 @@
         <v>108.01</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C28" s="4">
         <v>106.54</v>
@@ -1006,12 +997,12 @@
         <v>100.18</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C29" s="4">
         <v>94.1</v>
@@ -1023,12 +1014,12 @@
         <v>109.14</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C30" s="4">
         <v>116.46</v>
@@ -1040,12 +1031,12 @@
         <v>101.96</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C31" s="4">
         <v>169.14</v>
@@ -1057,12 +1048,12 @@
         <v>114.4</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C32" s="4">
         <v>105.86</v>
@@ -1074,12 +1065,12 @@
         <v>112.19</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C33" s="4">
         <v>77.86</v>
@@ -1091,12 +1082,12 @@
         <v>98.97</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C34" s="4">
         <v>83.36</v>
@@ -1108,12 +1099,12 @@
         <v>107.3</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C35" s="4">
         <v>111.28</v>
@@ -1125,12 +1116,12 @@
         <v>96.4</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C36" s="4">
         <v>111.74</v>
@@ -1142,12 +1133,12 @@
         <v>106.37</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C37" s="4">
         <v>95.04</v>
@@ -1159,12 +1150,12 @@
         <v>107.34</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C38" s="4">
         <v>100.48</v>
@@ -1176,12 +1167,12 @@
         <v>111.92</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C39" s="4">
         <v>73.58</v>
@@ -1193,12 +1184,12 @@
         <v>103.86</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C40" s="4">
         <v>106.6</v>
@@ -1210,12 +1201,12 @@
         <v>107.38</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C41" s="4">
         <v>76.040000000000006</v>
@@ -1227,12 +1218,12 @@
         <v>109.59</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C42" s="4">
         <v>104.22</v>
@@ -1244,12 +1235,12 @@
         <v>107.46</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C43" s="4">
         <v>103.78</v>
@@ -1261,12 +1252,12 @@
         <v>118.34</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C44" s="4">
         <v>55.32</v>
@@ -1278,12 +1269,12 @@
         <v>100.07</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C45" s="4">
         <v>156.46</v>
@@ -1295,12 +1286,12 @@
         <v>105.81</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C46" s="4">
         <v>120.98</v>
@@ -1312,12 +1303,12 @@
         <v>117.49</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C47" s="4">
         <v>112.02</v>
@@ -1329,12 +1320,12 @@
         <v>108.97</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C48" s="4">
         <v>168.48</v>
@@ -1346,12 +1337,12 @@
         <v>114.89</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C49" s="4">
         <v>143.30000000000001</v>
@@ -1363,12 +1354,12 @@
         <v>112.81</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C50" s="6">
         <v>140.12</v>
@@ -1379,16 +1370,13 @@
       <c r="E50" s="6">
         <v>121.81</v>
       </c>
-      <c r="F50" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C51" s="6">
         <v>108.34</v>
@@ -1399,16 +1387,13 @@
       <c r="E51" s="6">
         <v>101.2</v>
       </c>
-      <c r="F51" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C52" s="6">
         <v>123.8</v>
@@ -1419,16 +1404,13 @@
       <c r="E52" s="6">
         <v>105.49</v>
       </c>
-      <c r="F52" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C53" s="6">
         <v>113.24</v>
@@ -1439,16 +1421,13 @@
       <c r="E53" s="6">
         <v>111.17</v>
       </c>
-      <c r="F53" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C54" s="6">
         <v>129.06</v>
@@ -1459,16 +1438,13 @@
       <c r="E54" s="6">
         <v>105.38</v>
       </c>
-      <c r="F54" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="5" t="s">
-        <v>8</v>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C55" s="6">
         <v>85.66</v>
@@ -1479,16 +1455,13 @@
       <c r="E55" s="6">
         <v>119.22</v>
       </c>
-      <c r="F55" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="5" t="s">
-        <v>9</v>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C56" s="6">
         <v>115.3</v>
@@ -1499,16 +1472,13 @@
       <c r="E56" s="6">
         <v>108.3</v>
       </c>
-      <c r="F56" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C57" s="6">
         <v>88.06</v>
@@ -1519,16 +1489,13 @@
       <c r="E57" s="6">
         <v>103.14</v>
       </c>
-      <c r="F57" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C58" s="6">
         <v>141.24</v>
@@ -1539,16 +1506,13 @@
       <c r="E58" s="6">
         <v>117.67</v>
       </c>
-      <c r="F58" t="s">
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="C59" s="6">
         <v>126.1</v>
@@ -1559,16 +1523,13 @@
       <c r="E59" s="6">
         <v>107.35</v>
       </c>
-      <c r="F59" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C60" s="6">
         <v>128.74</v>
@@ -1579,16 +1540,13 @@
       <c r="E60" s="6">
         <v>105.91</v>
       </c>
-      <c r="F60" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C61" s="6">
         <v>103.34</v>
@@ -1599,11 +1557,249 @@
       <c r="E61" s="6">
         <v>105.37</v>
       </c>
-      <c r="F61" t="s">
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" s="4">
+        <v>90</v>
+      </c>
+      <c r="D62" s="4">
+        <v>107.22</v>
+      </c>
+      <c r="E62" s="4">
+        <v>100.07</v>
+      </c>
+      <c r="F62" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="B63" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="4">
+        <v>56.38</v>
+      </c>
+      <c r="D63" s="4">
+        <v>112.54</v>
+      </c>
+      <c r="E63" s="4">
+        <v>74.37</v>
+      </c>
+      <c r="F63" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C64" s="4">
+        <v>84.28</v>
+      </c>
+      <c r="D64" s="4">
+        <v>116.02</v>
+      </c>
+      <c r="E64" s="4">
+        <v>103.59</v>
+      </c>
+      <c r="F64" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C65" s="4">
+        <v>112.54</v>
+      </c>
+      <c r="D65" s="4">
+        <v>56.38</v>
+      </c>
+      <c r="E65" s="4">
+        <v>107.65</v>
+      </c>
+      <c r="F65" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C66" s="4">
+        <v>115.78</v>
+      </c>
+      <c r="D66" s="4">
+        <v>93.9</v>
+      </c>
+      <c r="E66" s="4">
+        <v>115.47</v>
+      </c>
+      <c r="F66" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C67" s="4">
+        <v>97.1</v>
+      </c>
+      <c r="D67" s="4">
+        <v>82.42</v>
+      </c>
+      <c r="E67" s="4">
+        <v>103.2</v>
+      </c>
+      <c r="F67" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C68" s="4">
+        <v>93.9</v>
+      </c>
+      <c r="D68" s="4">
+        <v>115.78</v>
+      </c>
+      <c r="E68" s="4">
+        <v>108.69</v>
+      </c>
+      <c r="F68" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C69" s="4">
+        <v>86.5</v>
+      </c>
+      <c r="D69" s="4">
+        <v>129.58000000000001</v>
+      </c>
+      <c r="E69" s="4">
+        <v>104.16</v>
+      </c>
+      <c r="F69" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C70" s="4">
+        <v>82.42</v>
+      </c>
+      <c r="D70" s="4">
+        <v>97.1</v>
+      </c>
+      <c r="E70" s="4">
+        <v>115.93</v>
+      </c>
+      <c r="F70" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C71" s="4">
+        <v>107.22</v>
+      </c>
+      <c r="D71" s="4">
+        <v>90</v>
+      </c>
+      <c r="E71" s="4">
+        <v>93.13</v>
+      </c>
+      <c r="F71" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C72" s="4">
+        <v>129.58000000000001</v>
+      </c>
+      <c r="D72" s="4">
+        <v>86.5</v>
+      </c>
+      <c r="E72" s="4">
+        <v>112.62</v>
+      </c>
+      <c r="F72" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C73" s="4">
+        <v>116.02</v>
+      </c>
+      <c r="D73" s="4">
+        <v>84.28</v>
+      </c>
+      <c r="E73" s="4">
+        <v>113.05</v>
+      </c>
+      <c r="F73" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{1686F8B2-D22C-A048-AC94-1D883AEA5A06}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>